<commit_message>
fix(get_commit) : correction d'un bug de duplication dans le get_commit
[6][DONE]
</commit_message>
<xml_diff>
--- a/Doc/journal_de_travail.xlsx
+++ b/Doc/journal_de_travail.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Tableau de bord" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -171,6 +171,699 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
@@ -282,7 +975,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -434,6 +1127,138 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="6" name="Chart 6"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="7" name="Chart 7"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId7"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="8" name="Chart 8"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId8"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -731,7 +1556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -897,31 +1722,430 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr"/>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>feat(jdt)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>[1]</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>feat(jdt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr"/>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>feat(gitignore) : création du gitignore</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>[4]</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>feat(gitignore) : création du gitignore</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>feat(tag) : création de la page de tagManagement</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>[27]</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>feat(tag) : création de la page de tagManagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>feat(library) : création de la page pour la liste des livres</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>[26]</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>feat(library) : création de la page pour la liste des livres</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>feat(read) : création de la page de lecture</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>[38]</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>feat(read) : création de la page de lecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>feat(model) : création des models</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>[18]</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>feat(model) : création des models</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>feat(viewModel) : création des viewMOdels</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>[83]</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>feat(viewModel) : création des viewMOdels  j'ai du utilisé de l'IA pour m'aider</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr"/>
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Total du jour</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>0h10 (10 min)</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>3h27 (207 min)</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>feat(service) création des services</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>[67]</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>feat(service) création des services   Bookservice: Le gestionnaire de livres TagService : Le gestionnaire de catégories</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>feat(resources) : mise des fichier de resources</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>[31]</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>feat(resources) : mise des fichier de resources</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>fix(backup) : mise des fichier de backup suite a un problème</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>[13]</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>fix(backup) : mise des fichier de backup suite a un problème"01/04/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>feat(gitignore) : création du gitignore</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>[4]</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>feat(gitignore) : création du gitignore</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>feat(tag) : création de la page de tagManagement</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>[27]</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>feat(tag) : création de la page de tagManagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>feat(library) : création de la page pour la liste des livres</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>[26]</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>feat(library) : création de la page pour la liste des livres</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>feat(read) : création de la page de lecture</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>[38]</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>feat(read) : création de la page de lecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>feat(model) : création des models</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>[18]</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>feat(model) : création des models</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr"/>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>feat(viewModel) : création des viewMOdels</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>[83]</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>feat(viewModel) : création des viewMOdels  j'ai du utilisé de l'IA pour m'aider</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr"/>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Total du jour</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>5h07 (307 min)</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr"/>
+      <c r="E29" s="4" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E11"/>
-  <mergeCells count="2">
+  <autoFilter ref="A1:E30"/>
+  <mergeCells count="4">
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A12:E12"/>
     <mergeCell ref="A8:E8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1008,7 +2232,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -1026,14 +2250,14 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
+        <v>207</v>
       </c>
       <c r="C3" t="n">
-        <v>0.17</v>
+        <v>3.45</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0h10</t>
+          <t>3h27</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -1043,7 +2267,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1h42</t>
+          <t>10h06</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1052,10 +2276,26 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>1.7</v>
+        <v>4.98</v>
       </c>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>307</v>
+      </c>
+      <c r="C4" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>5h07</t>
+        </is>
+      </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Moyenne / jour</t>
@@ -1063,8 +2303,16 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0h51</t>
-        </is>
+          <t>3h22</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>10.1</v>
       </c>
     </row>
     <row r="5">
@@ -1075,12 +2323,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>18/03/2026 (1h32)</t>
+          <t>01/04/2026 (5h07)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D3"/>
+  <autoFilter ref="A1:D4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(services) : création des services
[30][WIP]

j'ai pris du temps pour lancer sur le tél
</commit_message>
<xml_diff>
--- a/Doc/journal_de_travail.xlsx
+++ b/Doc/journal_de_travail.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Tableau de bord" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -281,6 +281,117 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
@@ -864,7 +975,6 @@
 
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -1009,6 +1119,14 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
           <cat>
             <numRef>
               <f>'Tableau de bord'!$A$2:$A$5</f>
@@ -1024,6 +1142,119 @@
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -1259,6 +1490,50 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId8"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="9" name="Chart 9"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId9"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="10" name="Chart 10"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId10"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1556,7 +1831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1976,7 +2251,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>fix(backup) : mise des fichier de backup suite a un problème"01/04/2026</t>
+          <t>fix(backup) : mise des fichier de backup suite a un problème</t>
         </is>
       </c>
     </row>
@@ -1984,12 +2259,12 @@
       <c r="A23" s="3" t="inlineStr"/>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>feat(gitignore) : création du gitignore</t>
+          <t>feat(jdt)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>[4]</t>
+          <t>[1]</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1999,7 +2274,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>feat(gitignore) : création du gitignore</t>
+          <t>feat(jdt)</t>
         </is>
       </c>
     </row>
@@ -2007,12 +2282,12 @@
       <c r="A24" s="3" t="inlineStr"/>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>feat(tag) : création de la page de tagManagement</t>
+          <t>feat(gitignore) : création du gitignore</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>[27]</t>
+          <t>[4]</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -2022,7 +2297,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>feat(tag) : création de la page de tagManagement</t>
+          <t>feat(gitignore) : création du gitignore</t>
         </is>
       </c>
     </row>
@@ -2030,12 +2305,12 @@
       <c r="A25" s="3" t="inlineStr"/>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>feat(library) : création de la page pour la liste des livres</t>
+          <t>feat(tag) : création de la page de tagManagement</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>[26]</t>
+          <t>[27]</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -2045,7 +2320,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>feat(library) : création de la page pour la liste des livres</t>
+          <t>feat(tag) : création de la page de tagManagement</t>
         </is>
       </c>
     </row>
@@ -2053,12 +2328,12 @@
       <c r="A26" s="3" t="inlineStr"/>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>feat(read) : création de la page de lecture</t>
+          <t>feat(library) : création de la page pour la liste des livres</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>[38]</t>
+          <t>[26]</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -2068,7 +2343,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>feat(read) : création de la page de lecture</t>
+          <t>feat(library) : création de la page pour la liste des livres</t>
         </is>
       </c>
     </row>
@@ -2076,12 +2351,12 @@
       <c r="A27" s="3" t="inlineStr"/>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>feat(model) : création des models</t>
+          <t>feat(read) : création de la page de lecture</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>[18]</t>
+          <t>[38]</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -2091,7 +2366,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>feat(model) : création des models</t>
+          <t>feat(read) : création de la page de lecture</t>
         </is>
       </c>
     </row>
@@ -2099,49 +2374,187 @@
       <c r="A28" s="3" t="inlineStr"/>
       <c r="B28" s="3" t="inlineStr">
         <is>
+          <t>feat(model) : création des models</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>[18]</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>feat(model) : création des models</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr"/>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
           <t>feat(viewModel) : création des viewMOdels</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>[83]</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>feat(viewModel) : création des viewMOdels  j'ai du utilisé de l'IA pour m'aider</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr"/>
-      <c r="B29" s="5" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr"/>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>fix(get_commit) : correction d'un bug de duplication dans le get_commit</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>[6]</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>fix(get_commit) : correction d'un bug de duplication dans le get_commit</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr"/>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>feat(reset) : suppression de tout pour recommencer car trop de bug</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>[38]</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>feat(reset) : suppression de tout pour recommencer car trop de bug   il y a vais trop de bug (environ 86) du coup j'ai décider de recommencer le projet</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr"/>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>feat(VS) : création du projet VS</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>[2]</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>feat(VS) : création du projet VS</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr"/>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>feat(Views) : création des views pour chaque page</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>[10]</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>feat(Views) : création des views pour chaque page</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr"/>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>feat(ViewModel) : création des viewModel pour le lien entre les views et les models</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>[10]</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>feat(ViewModel) : création des viewModel pour le lien entre les views et les models</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr"/>
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>Total du jour</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>5h07 (307 min)</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr"/>
-      <c r="E29" s="4" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr"/>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>6h14 (374 min)</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr"/>
+      <c r="E35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E30"/>
+  <autoFilter ref="A1:E36"/>
   <mergeCells count="4">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A19:E19"/>
@@ -2267,7 +2680,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>10h06</t>
+          <t>11h13</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -2286,14 +2699,14 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>307</v>
+        <v>374</v>
       </c>
       <c r="C4" t="n">
-        <v>5.12</v>
+        <v>6.23</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5h07</t>
+          <t>6h14</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -2303,7 +2716,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3h22</t>
+          <t>3h44</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -2312,7 +2725,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>10.1</v>
+        <v>11.22</v>
       </c>
     </row>
     <row r="5">
@@ -2323,7 +2736,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>01/04/2026 (5h07)</t>
+          <t>01/04/2026 (6h14)</t>
         </is>
       </c>
     </row>

</xml_diff>